<commit_message>
Daily NSE scan: 2026-10-14
</commit_message>
<xml_diff>
--- a/output/2026-10-14/enriched_analysis.xlsx
+++ b/output/2026-10-14/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.275</v>
+        <v>2.241</v>
       </c>
       <c r="W2" t="n">
-        <v>2770</v>
+        <v>2811</v>
       </c>
       <c r="X2" t="n">
-        <v>21.7</v>
+        <v>22</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,10 +1161,10 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.834</v>
+        <v>0.829</v>
       </c>
       <c r="W3" t="n">
-        <v>971</v>
+        <v>977</v>
       </c>
       <c r="X3" t="n">
         <v>136</v>
@@ -1396,10 +1396,10 @@
         <v>0.021</v>
       </c>
       <c r="W4" t="n">
-        <v>3406</v>
+        <v>3433</v>
       </c>
       <c r="X4" t="n">
-        <v>15.4</v>
+        <v>15.5</v>
       </c>
       <c r="Y4" t="n">
         <v>18</v>
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.045</v>
+        <v>0.044</v>
       </c>
       <c r="W5" t="n">
-        <v>2958</v>
+        <v>3031</v>
       </c>
       <c r="X5" t="n">
-        <v>10.2</v>
+        <v>10.4</v>
       </c>
       <c r="Y5" t="n">
         <v>36</v>
@@ -1857,13 +1857,13 @@
         </is>
       </c>
       <c r="V6" t="n">
-        <v>1.025</v>
+        <v>1.047</v>
       </c>
       <c r="W6" t="n">
-        <v>387</v>
+        <v>379</v>
       </c>
       <c r="X6" t="n">
-        <v>88.09999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="Y6" t="n">
         <v>111</v>
@@ -2089,13 +2089,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>0.51</v>
+        <v>0.513</v>
       </c>
       <c r="W7" t="n">
-        <v>568</v>
+        <v>565</v>
       </c>
       <c r="X7" t="n">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="Y7" t="n">
         <v>19</v>
@@ -2321,13 +2321,13 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>1.223</v>
+        <v>1.203</v>
       </c>
       <c r="W8" t="n">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="X8" t="n">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="Y8" t="n">
         <v>22</v>
@@ -2553,13 +2553,13 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>0.329</v>
+        <v>0.322</v>
       </c>
       <c r="W9" t="n">
-        <v>930</v>
+        <v>950</v>
       </c>
       <c r="X9" t="n">
-        <v>9.140000000000001</v>
+        <v>9.32</v>
       </c>
       <c r="Y9" t="n">
         <v>7</v>
@@ -2785,13 +2785,13 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>1.187</v>
+        <v>1.194</v>
       </c>
       <c r="W10" t="n">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="X10" t="n">
-        <v>7.17</v>
+        <v>7.14</v>
       </c>
       <c r="Y10" t="n">
         <v>17</v>
@@ -3017,13 +3017,13 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>1.457</v>
+        <v>1.443</v>
       </c>
       <c r="W11" t="n">
-        <v>9284</v>
+        <v>9377</v>
       </c>
       <c r="X11" t="n">
-        <v>1563</v>
+        <v>1579</v>
       </c>
       <c r="Y11" t="n">
         <v>-53</v>
@@ -3252,7 +3252,7 @@
         <v>0.047</v>
       </c>
       <c r="W12" t="n">
-        <v>15232</v>
+        <v>15249</v>
       </c>
       <c r="X12" t="n">
         <v>38.8</v>
@@ -3713,13 +3713,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>0.126</v>
+        <v>0.127</v>
       </c>
       <c r="W14" t="n">
-        <v>694</v>
+        <v>686</v>
       </c>
       <c r="X14" t="n">
-        <v>26.2</v>
+        <v>25.9</v>
       </c>
       <c r="Y14" t="n">
         <v>13</v>
@@ -3948,10 +3948,10 @@
         <v>0.049</v>
       </c>
       <c r="W15" t="n">
-        <v>1693</v>
+        <v>1673</v>
       </c>
       <c r="X15" t="n">
-        <v>22.8</v>
+        <v>22.5</v>
       </c>
       <c r="Y15" t="n">
         <v>55</v>
@@ -4177,13 +4177,13 @@
         </is>
       </c>
       <c r="V16" t="n">
-        <v>0.065</v>
+        <v>0.066</v>
       </c>
       <c r="W16" t="n">
-        <v>864</v>
+        <v>863</v>
       </c>
       <c r="X16" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="Y16" t="n">
         <v>19</v>
@@ -4407,10 +4407,10 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>1.981</v>
+        <v>1.959</v>
       </c>
       <c r="W17" t="n">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="n">
@@ -4637,13 +4637,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.175</v>
+        <v>0.174</v>
       </c>
       <c r="W18" t="n">
-        <v>969</v>
+        <v>978</v>
       </c>
       <c r="X18" t="n">
-        <v>39.8</v>
+        <v>40.2</v>
       </c>
       <c r="Y18" t="n">
         <v>2</v>
@@ -4869,13 +4869,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.241</v>
+        <v>0.233</v>
       </c>
       <c r="W19" t="n">
-        <v>1428</v>
+        <v>1476</v>
       </c>
       <c r="X19" t="n">
-        <v>24.3</v>
+        <v>25.1</v>
       </c>
       <c r="Y19" t="n">
         <v>8</v>
@@ -5099,13 +5099,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.132</v>
+        <v>0.126</v>
       </c>
       <c r="W20" t="n">
-        <v>2383</v>
+        <v>2494</v>
       </c>
       <c r="X20" t="n">
-        <v>20.9</v>
+        <v>21.8</v>
       </c>
       <c r="Y20" t="n">
         <v>-3</v>
@@ -5331,13 +5331,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="W21" t="n">
-        <v>2523</v>
+        <v>2542</v>
       </c>
       <c r="X21" t="n">
-        <v>20.7</v>
+        <v>20.8</v>
       </c>
       <c r="Y21" t="n">
         <v>8</v>
@@ -5563,13 +5563,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>3.179</v>
+        <v>3.144</v>
       </c>
       <c r="W22" t="n">
-        <v>619</v>
+        <v>626</v>
       </c>
       <c r="X22" t="n">
-        <v>18.7</v>
+        <v>18.9</v>
       </c>
       <c r="Y22" t="n">
         <v>30</v>
@@ -5792,10 +5792,10 @@
         <v>0.178</v>
       </c>
       <c r="W23" t="n">
-        <v>624</v>
+        <v>621</v>
       </c>
       <c r="X23" t="n">
-        <v>52.1</v>
+        <v>51.9</v>
       </c>
       <c r="Y23" t="n">
         <v>3</v>
@@ -6021,13 +6021,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.102</v>
+        <v>0.101</v>
       </c>
       <c r="W24" t="n">
-        <v>845</v>
+        <v>848</v>
       </c>
       <c r="X24" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="Y24" t="n">
         <v>17</v>
@@ -6247,13 +6247,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.139</v>
+        <v>0.135</v>
       </c>
       <c r="W25" t="n">
-        <v>1523</v>
+        <v>1568</v>
       </c>
       <c r="X25" t="n">
-        <v>15.2</v>
+        <v>15.6</v>
       </c>
       <c r="Y25" t="n">
         <v>152</v>
@@ -6479,13 +6479,13 @@
         </is>
       </c>
       <c r="V26" t="n">
-        <v>0.061</v>
+        <v>0.06</v>
       </c>
       <c r="W26" t="n">
-        <v>2088</v>
+        <v>2112</v>
       </c>
       <c r="X26" t="n">
-        <v>97</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="Y26" t="n">
         <v>13</v>
@@ -6711,13 +6711,13 @@
         </is>
       </c>
       <c r="V27" t="n">
-        <v>0.344</v>
+        <v>0.337</v>
       </c>
       <c r="W27" t="n">
-        <v>940</v>
+        <v>959</v>
       </c>
       <c r="X27" t="n">
-        <v>13.2</v>
+        <v>13.4</v>
       </c>
       <c r="Y27" t="n">
         <v>13</v>
@@ -6943,13 +6943,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.065</v>
+        <v>0.064</v>
       </c>
       <c r="W28" t="n">
-        <v>1712</v>
+        <v>1745</v>
       </c>
       <c r="X28" t="n">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="Y28" t="n">
         <v>-48</v>
@@ -7175,13 +7175,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.068</v>
       </c>
       <c r="W29" t="n">
-        <v>1588</v>
+        <v>1628</v>
       </c>
       <c r="X29" t="n">
-        <v>36.4</v>
+        <v>37.4</v>
       </c>
       <c r="Y29" t="n">
         <v>20</v>
@@ -7407,13 +7407,13 @@
         </is>
       </c>
       <c r="V30" t="n">
-        <v>0.32</v>
+        <v>0.318</v>
       </c>
       <c r="W30" t="n">
-        <v>59404</v>
+        <v>59791</v>
       </c>
       <c r="X30" t="n">
-        <v>22.2</v>
+        <v>22.4</v>
       </c>
       <c r="Y30" t="n">
         <v>5</v>
@@ -7639,13 +7639,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.542</v>
+        <v>0.54</v>
       </c>
       <c r="W31" t="n">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="X31" t="n">
-        <v>16.1</v>
+        <v>16.2</v>
       </c>
       <c r="Y31" t="n">
         <v>13</v>
@@ -7874,10 +7874,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W32" t="n">
-        <v>55508</v>
+        <v>55776</v>
       </c>
       <c r="X32" t="n">
-        <v>47</v>
+        <v>47.2</v>
       </c>
       <c r="Y32" t="n">
         <v>5</v>
@@ -8106,7 +8106,7 @@
         <v>0.08599999999999999</v>
       </c>
       <c r="W33" t="n">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="X33" t="n">
         <v>10.8</v>
@@ -8335,13 +8335,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>1.633</v>
+        <v>1.597</v>
       </c>
       <c r="W34" t="n">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="X34" t="n">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="Y34" t="n">
         <v>-14</v>
@@ -8567,13 +8567,13 @@
         </is>
       </c>
       <c r="V35" t="n">
-        <v>0.16</v>
+        <v>0.153</v>
       </c>
       <c r="W35" t="n">
-        <v>3986</v>
+        <v>4189</v>
       </c>
       <c r="X35" t="n">
-        <v>7.51</v>
+        <v>7.9</v>
       </c>
       <c r="Y35" t="n">
         <v>2</v>
@@ -8799,13 +8799,13 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>1.102</v>
+        <v>1.12</v>
       </c>
       <c r="W36" t="n">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="X36" t="n">
-        <v>5.27</v>
+        <v>5.17</v>
       </c>
       <c r="Y36" t="n">
         <v>31</v>
@@ -9027,13 +9027,13 @@
         </is>
       </c>
       <c r="V37" t="n">
-        <v>0.263</v>
+        <v>0.26</v>
       </c>
       <c r="W37" t="n">
-        <v>990</v>
+        <v>1002</v>
       </c>
       <c r="X37" t="n">
-        <v>26.9</v>
+        <v>27.3</v>
       </c>
       <c r="Y37" t="n">
         <v>9</v>
@@ -9261,7 +9261,7 @@
       <c r="V38" t="inlineStr"/>
       <c r="W38" t="inlineStr"/>
       <c r="X38" t="n">
-        <v>5.87</v>
+        <v>5.58</v>
       </c>
       <c r="Y38" t="n">
         <v>-68</v>
@@ -9487,13 +9487,13 @@
         </is>
       </c>
       <c r="V39" t="n">
-        <v>1.075</v>
+        <v>1.082</v>
       </c>
       <c r="W39" t="n">
-        <v>1849</v>
+        <v>1838</v>
       </c>
       <c r="X39" t="n">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="Y39" t="n">
         <v>12</v>
@@ -9722,10 +9722,10 @@
         <v>0.01</v>
       </c>
       <c r="W40" t="n">
-        <v>14720</v>
+        <v>15097</v>
       </c>
       <c r="X40" t="n">
-        <v>13.6</v>
+        <v>13.9</v>
       </c>
       <c r="Y40" t="n">
         <v>28</v>
@@ -9951,13 +9951,13 @@
         </is>
       </c>
       <c r="V41" t="n">
-        <v>0.33</v>
+        <v>0.325</v>
       </c>
       <c r="W41" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="X41" t="n">
-        <v>23.3</v>
+        <v>23.6</v>
       </c>
       <c r="Y41" t="n">
         <v>12</v>
@@ -10186,10 +10186,10 @@
         <v>0.004</v>
       </c>
       <c r="W42" t="n">
-        <v>49527</v>
+        <v>47866</v>
       </c>
       <c r="X42" t="n">
-        <v>367</v>
+        <v>355</v>
       </c>
       <c r="Y42" t="n">
         <v>26</v>
@@ -10418,10 +10418,10 @@
         <v>0.374</v>
       </c>
       <c r="W43" t="n">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="X43" t="n">
-        <v>53.5</v>
+        <v>53.6</v>
       </c>
       <c r="Y43" t="n">
         <v>21</v>
@@ -10879,10 +10879,10 @@
         </is>
       </c>
       <c r="V45" t="n">
-        <v>1.876</v>
+        <v>1.845</v>
       </c>
       <c r="W45" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="X45" t="inlineStr"/>
       <c r="Y45" t="n">
@@ -11109,13 +11109,13 @@
         </is>
       </c>
       <c r="V46" t="n">
-        <v>0.524</v>
+        <v>0.52</v>
       </c>
       <c r="W46" t="n">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="X46" t="n">
-        <v>35.3</v>
+        <v>35.6</v>
       </c>
       <c r="Y46" t="n">
         <v>21</v>
@@ -11344,10 +11344,10 @@
         <v>0.042</v>
       </c>
       <c r="W47" t="n">
-        <v>1646</v>
+        <v>1633</v>
       </c>
       <c r="X47" t="n">
-        <v>21.5</v>
+        <v>21.3</v>
       </c>
       <c r="Y47" t="n">
         <v>10</v>
@@ -11573,10 +11573,10 @@
         </is>
       </c>
       <c r="V48" t="n">
-        <v>4.621</v>
+        <v>4.437</v>
       </c>
       <c r="W48" t="n">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="X48" t="inlineStr"/>
       <c r="Y48" t="n">
@@ -11803,13 +11803,13 @@
         </is>
       </c>
       <c r="V49" t="n">
-        <v>0.512</v>
+        <v>0.509</v>
       </c>
       <c r="W49" t="n">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="X49" t="n">
-        <v>36.4</v>
+        <v>36.6</v>
       </c>
       <c r="Y49" t="n">
         <v>-44</v>
@@ -11963,16 +11963,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tiger Logistics (India) Limited</t>
+          <t>TRUALT BIOENERGY LIMITED</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -11980,40 +11980,40 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F50" t="n">
-        <v>4</v>
+        <v>-3</v>
       </c>
       <c r="G50" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H50" t="n">
-        <v>-1</v>
+        <v>-16</v>
       </c>
       <c r="I50" t="n">
-        <v>24.27</v>
+        <v>447.2</v>
       </c>
       <c r="J50" t="n">
-        <v>27.53</v>
+        <v>349.57</v>
       </c>
       <c r="K50" t="n">
-        <v>-11.8</v>
+        <v>27.9</v>
       </c>
       <c r="L50" t="n">
-        <v>61.81</v>
+        <v>70.55</v>
       </c>
       <c r="M50" t="n">
-        <v>0.65</v>
+        <v>31.6</v>
       </c>
       <c r="N50" t="n">
-        <v>6470400</v>
+        <v>315995536</v>
       </c>
       <c r="O50" t="n">
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>6470400</v>
+        <v>315995536</v>
       </c>
       <c r="Q50" t="n">
         <v>0</v>
@@ -12027,7 +12027,7 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="U50" t="inlineStr">
         <is>
@@ -12035,52 +12035,52 @@
         </is>
       </c>
       <c r="V50" t="n">
-        <v>0.252</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="W50" t="n">
-        <v>257</v>
+        <v>3907</v>
       </c>
       <c r="X50" t="n">
-        <v>13.5</v>
+        <v>27.3</v>
       </c>
       <c r="Y50" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="Z50" t="n">
-        <v>2.79</v>
+        <v>127</v>
       </c>
       <c r="AA50" t="n">
-        <v>-30</v>
+        <v>-14</v>
       </c>
       <c r="AB50" t="n">
-        <v>0.21</v>
+        <v>6.41</v>
       </c>
       <c r="AC50" t="n">
-        <v>18</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="AD50" t="n">
-        <v>0.32</v>
+        <v>1.05</v>
       </c>
       <c r="AE50" t="b">
         <v>0</v>
       </c>
       <c r="AF50" t="n">
-        <v>1.83</v>
+        <v>21</v>
       </c>
       <c r="AG50" t="n">
-        <v>27.11</v>
+        <v>443.07</v>
       </c>
       <c r="AH50" t="n">
-        <v>31.44</v>
+        <v>433.75</v>
       </c>
       <c r="AI50" t="n">
-        <v>-19</v>
+        <v>7.2</v>
       </c>
       <c r="AJ50" t="n">
-        <v>27.53361702127659</v>
+        <v>349.5746258337085</v>
       </c>
       <c r="AK50" t="n">
-        <v>-11.9</v>
+        <v>27.9</v>
       </c>
       <c r="AL50" t="inlineStr">
         <is>
@@ -12094,12 +12094,12 @@
       </c>
       <c r="AN50" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO50" t="inlineStr">
         <is>
-          <t>19-08-2026</t>
+          <t>05-08-2026</t>
         </is>
       </c>
       <c r="AP50" t="inlineStr">
@@ -12108,10 +12108,10 @@
         </is>
       </c>
       <c r="AQ50" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="AR50" t="n">
-        <v>56</v>
+        <v>70</v>
       </c>
       <c r="AS50" t="n">
         <v>14</v>
@@ -12126,25 +12126,25 @@
         <v>6</v>
       </c>
       <c r="AW50" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AX50" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AY50" t="n">
         <v>0</v>
       </c>
       <c r="AZ50" t="n">
-        <v>925400</v>
+        <v>464</v>
       </c>
       <c r="BA50" t="n">
-        <v>4267650</v>
+        <v>213764633</v>
       </c>
       <c r="BB50" t="n">
-        <v>6470400</v>
+        <v>213764633</v>
       </c>
       <c r="BC50" t="n">
-        <v>6470400</v>
+        <v>315995536</v>
       </c>
       <c r="BD50" t="n">
         <v>0</v>
@@ -12180,7 +12180,7 @@
         <v>0</v>
       </c>
       <c r="BO50" t="n">
-        <v>4267650</v>
+        <v>213764633</v>
       </c>
       <c r="BP50" t="n">
         <v>1</v>
@@ -12195,12 +12195,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TRUALT</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TRUALT BIOENERGY LIMITED</t>
+          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -12212,107 +12212,103 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F51" t="n">
-        <v>-3</v>
+        <v>1</v>
       </c>
       <c r="G51" t="n">
+        <v>5</v>
+      </c>
+      <c r="H51" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I51" t="n">
+        <v>12.44</v>
+      </c>
+      <c r="J51" t="n">
+        <v>12.86</v>
+      </c>
+      <c r="K51" t="n">
+        <v>-3.3</v>
+      </c>
+      <c r="L51" t="n">
+        <v>69.12</v>
+      </c>
+      <c r="M51" t="n">
+        <v>2.35</v>
+      </c>
+      <c r="N51" t="n">
+        <v>23479616</v>
+      </c>
+      <c r="O51" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" t="n">
+        <v>23479616</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S51" t="b">
+        <v>0</v>
+      </c>
+      <c r="T51" t="n">
         <v>25</v>
       </c>
-      <c r="H51" t="n">
-        <v>-16</v>
-      </c>
-      <c r="I51" t="n">
-        <v>447.2</v>
-      </c>
-      <c r="J51" t="n">
-        <v>349.57</v>
-      </c>
-      <c r="K51" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="L51" t="n">
-        <v>70.55</v>
-      </c>
-      <c r="M51" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="N51" t="n">
-        <v>315995536</v>
-      </c>
-      <c r="O51" t="n">
-        <v>0</v>
-      </c>
-      <c r="P51" t="n">
-        <v>315995536</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>0</v>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S51" t="b">
-        <v>0</v>
-      </c>
-      <c r="T51" t="n">
-        <v>11</v>
-      </c>
       <c r="U51" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="V51" t="n">
-        <v>0.824</v>
+        <v>0.695</v>
       </c>
       <c r="W51" t="n">
-        <v>3837</v>
+        <v>338</v>
       </c>
       <c r="X51" t="n">
-        <v>26.8</v>
+        <v>1091</v>
       </c>
       <c r="Y51" t="n">
-        <v>2</v>
-      </c>
-      <c r="Z51" t="n">
-        <v>127</v>
-      </c>
+        <v>-61</v>
+      </c>
+      <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="n">
-        <v>-14</v>
+        <v>-98</v>
       </c>
       <c r="AB51" t="n">
-        <v>6.41</v>
+        <v>0.01</v>
       </c>
       <c r="AC51" t="n">
-        <v>9.890000000000001</v>
+        <v>2.46</v>
       </c>
       <c r="AD51" t="n">
-        <v>1.05</v>
+        <v>0.44</v>
       </c>
       <c r="AE51" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF51" t="n">
-        <v>21</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="AF51" t="inlineStr"/>
       <c r="AG51" t="n">
-        <v>443.07</v>
+        <v>12.83</v>
       </c>
       <c r="AH51" t="n">
-        <v>433.75</v>
+        <v>12.91</v>
       </c>
       <c r="AI51" t="n">
-        <v>7.2</v>
+        <v>0.6</v>
       </c>
       <c r="AJ51" t="n">
-        <v>349.5746258337085</v>
+        <v>12.85608234597773</v>
       </c>
       <c r="AK51" t="n">
-        <v>27.9</v>
+        <v>-3.2</v>
       </c>
       <c r="AL51" t="inlineStr">
         <is>
@@ -12326,57 +12322,57 @@
       </c>
       <c r="AN51" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO51" t="inlineStr">
         <is>
-          <t>05-08-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="AP51" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AQ51" t="n">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="AR51" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="AS51" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="AT51" t="n">
         <v>0</v>
       </c>
       <c r="AU51" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV51" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AW51" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="AX51" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="AY51" t="n">
         <v>0</v>
       </c>
       <c r="AZ51" t="n">
-        <v>464</v>
+        <v>0</v>
       </c>
       <c r="BA51" t="n">
-        <v>213764633</v>
+        <v>2496337</v>
       </c>
       <c r="BB51" t="n">
-        <v>213764633</v>
+        <v>16559572</v>
       </c>
       <c r="BC51" t="n">
-        <v>315995536</v>
+        <v>23479616</v>
       </c>
       <c r="BD51" t="n">
         <v>0</v>
@@ -12412,7 +12408,7 @@
         <v>0</v>
       </c>
       <c r="BO51" t="n">
-        <v>213764633</v>
+        <v>2496337</v>
       </c>
       <c r="BP51" t="n">
         <v>1</v>
@@ -12427,12 +12423,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>SHAKTIPUMP</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
+          <t>SHAKTI PUMPS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -12444,40 +12440,40 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G52" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H52" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>12.44</v>
+        <v>424.45</v>
       </c>
       <c r="J52" t="n">
-        <v>12.86</v>
+        <v>473.17</v>
       </c>
       <c r="K52" t="n">
-        <v>-3.3</v>
+        <v>-10.3</v>
       </c>
       <c r="L52" t="n">
-        <v>69.12</v>
+        <v>56.22</v>
       </c>
       <c r="M52" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
       <c r="N52" t="n">
-        <v>23479616</v>
+        <v>23279819</v>
       </c>
       <c r="O52" t="n">
         <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>23479616</v>
+        <v>23279819</v>
       </c>
       <c r="Q52" t="n">
         <v>0</v>
@@ -12491,56 +12487,60 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="U52" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="V52" t="n">
-        <v>0.669</v>
+        <v>0.044</v>
       </c>
       <c r="W52" t="n">
-        <v>351</v>
+        <v>5241</v>
       </c>
       <c r="X52" t="n">
-        <v>1132</v>
+        <v>27.2</v>
       </c>
       <c r="Y52" t="n">
-        <v>-61</v>
-      </c>
-      <c r="Z52" t="inlineStr"/>
+        <v>13</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>59</v>
+      </c>
       <c r="AA52" t="n">
-        <v>-98</v>
+        <v>-52</v>
       </c>
       <c r="AB52" t="n">
-        <v>0.01</v>
+        <v>3.48</v>
       </c>
       <c r="AC52" t="n">
-        <v>2.46</v>
+        <v>24.3</v>
       </c>
       <c r="AD52" t="n">
-        <v>0.44</v>
+        <v>0.26</v>
       </c>
       <c r="AE52" t="b">
         <v>1</v>
       </c>
-      <c r="AF52" t="inlineStr"/>
+      <c r="AF52" t="n">
+        <v>7</v>
+      </c>
       <c r="AG52" t="n">
-        <v>12.83</v>
+        <v>479.42</v>
       </c>
       <c r="AH52" t="n">
-        <v>12.91</v>
+        <v>548.23</v>
       </c>
       <c r="AI52" t="n">
-        <v>0.6</v>
+        <v>-16.8</v>
       </c>
       <c r="AJ52" t="n">
-        <v>12.85608234597773</v>
+        <v>473.1670528455285</v>
       </c>
       <c r="AK52" t="n">
-        <v>-3.2</v>
+        <v>-10.3</v>
       </c>
       <c r="AL52" t="inlineStr">
         <is>
@@ -12559,22 +12559,22 @@
       </c>
       <c r="AO52" t="inlineStr">
         <is>
-          <t>10-08-2026</t>
+          <t>08-09-2026</t>
         </is>
       </c>
       <c r="AP52" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
       <c r="AQ52" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="AR52" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="AS52" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="AT52" t="n">
         <v>0</v>
@@ -12583,13 +12583,13 @@
         <v>0</v>
       </c>
       <c r="AV52" t="n">
+        <v>2</v>
+      </c>
+      <c r="AW52" t="n">
         <v>4</v>
       </c>
-      <c r="AW52" t="n">
-        <v>22</v>
-      </c>
       <c r="AX52" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="AY52" t="n">
         <v>0</v>
@@ -12598,13 +12598,13 @@
         <v>0</v>
       </c>
       <c r="BA52" t="n">
-        <v>2496337</v>
+        <v>11585069</v>
       </c>
       <c r="BB52" t="n">
-        <v>16559572</v>
+        <v>23279819</v>
       </c>
       <c r="BC52" t="n">
-        <v>23479616</v>
+        <v>23279819</v>
       </c>
       <c r="BD52" t="n">
         <v>0</v>
@@ -12640,10 +12640,10 @@
         <v>0</v>
       </c>
       <c r="BO52" t="n">
-        <v>2496337</v>
+        <v>11585069</v>
       </c>
       <c r="BP52" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BQ52" t="n">
         <v>0</v>
@@ -12655,12 +12655,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SHAKTIPUMP</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SHAKTI PUMPS (INDIA) LIMITED</t>
+          <t>Dangee Dums Limited</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -12672,40 +12672,40 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F53" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G53" t="n">
         <v>12</v>
       </c>
-      <c r="G53" t="n">
-        <v>0</v>
-      </c>
       <c r="H53" t="n">
         <v>0</v>
       </c>
       <c r="I53" t="n">
-        <v>424.45</v>
+        <v>3.26</v>
       </c>
       <c r="J53" t="n">
-        <v>473.17</v>
+        <v>2.82</v>
       </c>
       <c r="K53" t="n">
-        <v>-10.3</v>
+        <v>15.6</v>
       </c>
       <c r="L53" t="n">
-        <v>56.22</v>
+        <v>64.45</v>
       </c>
       <c r="M53" t="n">
-        <v>2.33</v>
+        <v>2.02</v>
       </c>
       <c r="N53" t="n">
-        <v>23279819</v>
+        <v>20159573</v>
       </c>
       <c r="O53" t="n">
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>23279819</v>
+        <v>20159573</v>
       </c>
       <c r="Q53" t="n">
         <v>0</v>
@@ -12719,60 +12719,54 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="U53" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
-        </is>
-      </c>
-      <c r="V53" t="n">
-        <v>0.044</v>
-      </c>
-      <c r="W53" t="n">
-        <v>5238</v>
-      </c>
-      <c r="X53" t="n">
-        <v>27.2</v>
-      </c>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr"/>
+      <c r="W53" t="inlineStr"/>
+      <c r="X53" t="inlineStr"/>
       <c r="Y53" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="Z53" t="n">
-        <v>59</v>
+        <v>0.98</v>
       </c>
       <c r="AA53" t="n">
-        <v>-52</v>
+        <v>-86</v>
       </c>
       <c r="AB53" t="n">
-        <v>3.48</v>
+        <v>-0.03</v>
       </c>
       <c r="AC53" t="n">
-        <v>24.3</v>
+        <v>2.27</v>
       </c>
       <c r="AD53" t="n">
-        <v>0.26</v>
+        <v>1.58</v>
       </c>
       <c r="AE53" t="b">
         <v>1</v>
       </c>
       <c r="AF53" t="n">
-        <v>7</v>
+        <v>14.22</v>
       </c>
       <c r="AG53" t="n">
-        <v>479.42</v>
+        <v>2.91</v>
       </c>
       <c r="AH53" t="n">
-        <v>548.23</v>
+        <v>3.16</v>
       </c>
       <c r="AI53" t="n">
-        <v>-16.8</v>
+        <v>-3.6</v>
       </c>
       <c r="AJ53" t="n">
-        <v>473.1670528455285</v>
+        <v>2.817550384346611</v>
       </c>
       <c r="AK53" t="n">
-        <v>-10.3</v>
+        <v>15.7</v>
       </c>
       <c r="AL53" t="inlineStr">
         <is>
@@ -12781,32 +12775,32 @@
       </c>
       <c r="AM53" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN53" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO53" t="inlineStr">
         <is>
-          <t>08-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AP53" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AQ53" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="AR53" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="AS53" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="AT53" t="n">
         <v>0</v>
@@ -12815,13 +12809,13 @@
         <v>0</v>
       </c>
       <c r="AV53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AW53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AX53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AY53" t="n">
         <v>0</v>
@@ -12830,13 +12824,13 @@
         <v>0</v>
       </c>
       <c r="BA53" t="n">
-        <v>11585069</v>
+        <v>20159573</v>
       </c>
       <c r="BB53" t="n">
-        <v>23279819</v>
+        <v>20159573</v>
       </c>
       <c r="BC53" t="n">
-        <v>23279819</v>
+        <v>20159573</v>
       </c>
       <c r="BD53" t="n">
         <v>0</v>
@@ -12872,10 +12866,10 @@
         <v>0</v>
       </c>
       <c r="BO53" t="n">
-        <v>11585069</v>
+        <v>20159573</v>
       </c>
       <c r="BP53" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="BQ53" t="n">
         <v>0</v>
@@ -12887,182 +12881,188 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dangee Dums Limited</t>
+          <t>Tiger Logistics (India) Limited</t>
         </is>
       </c>
       <c r="C54" t="n">
+        <v>5</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>5</v>
+      </c>
+      <c r="F54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" t="n">
+        <v>-1</v>
+      </c>
+      <c r="I54" t="n">
+        <v>24.27</v>
+      </c>
+      <c r="J54" t="n">
+        <v>27.53</v>
+      </c>
+      <c r="K54" t="n">
+        <v>-11.8</v>
+      </c>
+      <c r="L54" t="n">
+        <v>61.81</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="N54" t="n">
+        <v>6470400</v>
+      </c>
+      <c r="O54" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" t="n">
+        <v>6470400</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Net Buying</t>
+        </is>
+      </c>
+      <c r="S54" t="b">
+        <v>0</v>
+      </c>
+      <c r="T54" t="n">
+        <v>9</v>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="V54" t="n">
+        <v>0.241</v>
+      </c>
+      <c r="W54" t="n">
+        <v>268</v>
+      </c>
+      <c r="X54" t="n">
+        <v>14.1</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>16</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>2.79</v>
+      </c>
+      <c r="AA54" t="n">
+        <v>-30</v>
+      </c>
+      <c r="AB54" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>18</v>
+      </c>
+      <c r="AD54" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="AE54" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF54" t="n">
+        <v>1.83</v>
+      </c>
+      <c r="AG54" t="n">
+        <v>27.11</v>
+      </c>
+      <c r="AH54" t="n">
+        <v>31.44</v>
+      </c>
+      <c r="AI54" t="n">
+        <v>-19</v>
+      </c>
+      <c r="AJ54" t="n">
+        <v>27.53361702127659</v>
+      </c>
+      <c r="AK54" t="n">
+        <v>-11.9</v>
+      </c>
+      <c r="AL54" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AM54" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AN54" t="inlineStr">
+        <is>
+          <t>Confirmed Accumulation</t>
+        </is>
+      </c>
+      <c r="AO54" t="inlineStr">
+        <is>
+          <t>19-08-2026</t>
+        </is>
+      </c>
+      <c r="AP54" t="inlineStr">
+        <is>
+          <t>30-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ54" t="n">
+        <v>42</v>
+      </c>
+      <c r="AR54" t="n">
+        <v>56</v>
+      </c>
+      <c r="AS54" t="n">
+        <v>14</v>
+      </c>
+      <c r="AT54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV54" t="n">
         <v>6</v>
       </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-      <c r="E54" t="n">
-        <v>3</v>
-      </c>
-      <c r="F54" t="n">
-        <v>-2</v>
-      </c>
-      <c r="G54" t="n">
-        <v>12</v>
-      </c>
-      <c r="H54" t="n">
-        <v>0</v>
-      </c>
-      <c r="I54" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="J54" t="n">
-        <v>2.82</v>
-      </c>
-      <c r="K54" t="n">
-        <v>15.6</v>
-      </c>
-      <c r="L54" t="n">
-        <v>64.45</v>
-      </c>
-      <c r="M54" t="n">
-        <v>2.02</v>
-      </c>
-      <c r="N54" t="n">
-        <v>20159573</v>
-      </c>
-      <c r="O54" t="n">
-        <v>0</v>
-      </c>
-      <c r="P54" t="n">
-        <v>20159573</v>
-      </c>
-      <c r="Q54" t="n">
-        <v>0</v>
-      </c>
-      <c r="R54" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S54" t="b">
-        <v>0</v>
-      </c>
-      <c r="T54" t="n">
-        <v>1</v>
-      </c>
-      <c r="U54" t="inlineStr">
-        <is>
-          <t>24-09-2026</t>
-        </is>
-      </c>
-      <c r="V54" t="inlineStr"/>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
-      <c r="Y54" t="n">
-        <v>10</v>
-      </c>
-      <c r="Z54" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="AA54" t="n">
-        <v>-86</v>
-      </c>
-      <c r="AB54" t="n">
-        <v>-0.03</v>
-      </c>
-      <c r="AC54" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="AD54" t="n">
-        <v>1.58</v>
-      </c>
-      <c r="AE54" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF54" t="n">
-        <v>14.22</v>
-      </c>
-      <c r="AG54" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="AH54" t="n">
-        <v>3.16</v>
-      </c>
-      <c r="AI54" t="n">
-        <v>-3.6</v>
-      </c>
-      <c r="AJ54" t="n">
-        <v>2.817550384346611</v>
-      </c>
-      <c r="AK54" t="n">
-        <v>15.7</v>
-      </c>
-      <c r="AL54" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AM54" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN54" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AO54" t="inlineStr">
-        <is>
-          <t>24-09-2026</t>
-        </is>
-      </c>
-      <c r="AP54" t="inlineStr">
-        <is>
-          <t>24-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ54" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR54" t="n">
-        <v>20</v>
-      </c>
-      <c r="AS54" t="n">
-        <v>20</v>
-      </c>
-      <c r="AT54" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU54" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV54" t="n">
-        <v>1</v>
-      </c>
       <c r="AW54" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="AX54" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="AY54" t="n">
         <v>0</v>
       </c>
       <c r="AZ54" t="n">
-        <v>0</v>
+        <v>925400</v>
       </c>
       <c r="BA54" t="n">
-        <v>20159573</v>
+        <v>4267650</v>
       </c>
       <c r="BB54" t="n">
-        <v>20159573</v>
+        <v>6470400</v>
       </c>
       <c r="BC54" t="n">
-        <v>20159573</v>
+        <v>6470400</v>
       </c>
       <c r="BD54" t="n">
         <v>0</v>
@@ -13098,7 +13098,7 @@
         <v>0</v>
       </c>
       <c r="BO54" t="n">
-        <v>20159573</v>
+        <v>4267650</v>
       </c>
       <c r="BP54" t="n">
         <v>1</v>
@@ -13185,13 +13185,13 @@
         </is>
       </c>
       <c r="V55" t="n">
-        <v>0.231</v>
+        <v>0.229</v>
       </c>
       <c r="W55" t="n">
-        <v>1730</v>
+        <v>1743</v>
       </c>
       <c r="X55" t="n">
-        <v>18.3</v>
+        <v>18.4</v>
       </c>
       <c r="Y55" t="n">
         <v>-3</v>
@@ -13420,7 +13420,7 @@
         <v>0.042</v>
       </c>
       <c r="W56" t="n">
-        <v>3213</v>
+        <v>3224</v>
       </c>
       <c r="X56" t="n">
         <v>19.1</v>
@@ -13649,13 +13649,13 @@
         </is>
       </c>
       <c r="V57" t="n">
-        <v>0.372</v>
+        <v>0.366</v>
       </c>
       <c r="W57" t="n">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="X57" t="n">
-        <v>93.09999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="Y57" t="n">
         <v>246</v>
@@ -13881,13 +13881,13 @@
         </is>
       </c>
       <c r="V58" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
       <c r="W58" t="n">
-        <v>7493</v>
+        <v>7682</v>
       </c>
       <c r="X58" t="n">
-        <v>30</v>
+        <v>30.8</v>
       </c>
       <c r="Y58" t="n">
         <v>25</v>
@@ -14109,13 +14109,13 @@
         </is>
       </c>
       <c r="V59" t="n">
-        <v>0.332</v>
+        <v>0.328</v>
       </c>
       <c r="W59" t="n">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="X59" t="n">
-        <v>57.7</v>
+        <v>58.4</v>
       </c>
       <c r="Y59" t="n">
         <v>13</v>
@@ -14573,13 +14573,13 @@
         </is>
       </c>
       <c r="V61" t="n">
-        <v>0.198</v>
+        <v>0.2</v>
       </c>
       <c r="W61" t="n">
-        <v>500</v>
+        <v>494</v>
       </c>
       <c r="X61" t="n">
-        <v>14.6</v>
+        <v>14.4</v>
       </c>
       <c r="Y61" t="n">
         <v>-1</v>
@@ -14805,13 +14805,13 @@
         </is>
       </c>
       <c r="V62" t="n">
-        <v>0.483</v>
+        <v>0.474</v>
       </c>
       <c r="W62" t="n">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="X62" t="n">
-        <v>41.6</v>
+        <v>42.4</v>
       </c>
       <c r="Y62" t="n">
         <v>6</v>
@@ -15272,10 +15272,10 @@
         <v>0</v>
       </c>
       <c r="W64" t="n">
-        <v>5218</v>
+        <v>5334</v>
       </c>
       <c r="X64" t="n">
-        <v>12.2</v>
+        <v>12.5</v>
       </c>
       <c r="Y64" t="n">
         <v>26</v>
@@ -15501,13 +15501,13 @@
         </is>
       </c>
       <c r="V65" t="n">
-        <v>0.101</v>
+        <v>0.105</v>
       </c>
       <c r="W65" t="n">
-        <v>491</v>
+        <v>471</v>
       </c>
       <c r="X65" t="n">
-        <v>7.93</v>
+        <v>7.61</v>
       </c>
       <c r="Y65" t="n">
         <v>118</v>
@@ -15729,13 +15729,13 @@
         </is>
       </c>
       <c r="V66" t="n">
-        <v>0.145</v>
+        <v>0.143</v>
       </c>
       <c r="W66" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="X66" t="n">
-        <v>32.2</v>
+        <v>32.5</v>
       </c>
       <c r="Y66" t="n">
         <v>19</v>
@@ -15964,7 +15964,7 @@
         <v>0.011</v>
       </c>
       <c r="W67" t="n">
-        <v>3962</v>
+        <v>4006</v>
       </c>
       <c r="X67" t="inlineStr"/>
       <c r="Y67" t="n">
@@ -16194,7 +16194,7 @@
         <v>0.074</v>
       </c>
       <c r="W68" t="n">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="X68" t="n">
         <v>13.5</v>
@@ -16423,13 +16423,13 @@
         </is>
       </c>
       <c r="V69" t="n">
-        <v>0.1</v>
+        <v>0.097</v>
       </c>
       <c r="W69" t="n">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="X69" t="n">
-        <v>27.5</v>
+        <v>28.2</v>
       </c>
       <c r="Y69" t="n">
         <v>24</v>
@@ -16658,10 +16658,10 @@
         <v>0</v>
       </c>
       <c r="W70" t="n">
-        <v>3531</v>
+        <v>3520</v>
       </c>
       <c r="X70" t="n">
-        <v>45.9</v>
+        <v>45.8</v>
       </c>
       <c r="Y70" t="n">
         <v>5</v>
@@ -16890,10 +16890,10 @@
         <v>0.035</v>
       </c>
       <c r="W71" t="n">
-        <v>1395</v>
+        <v>1399</v>
       </c>
       <c r="X71" t="n">
-        <v>24.4</v>
+        <v>24.5</v>
       </c>
       <c r="Y71" t="n">
         <v>11</v>
@@ -17122,10 +17122,10 @@
         <v>0.003</v>
       </c>
       <c r="W72" t="n">
-        <v>12669</v>
+        <v>12885</v>
       </c>
       <c r="X72" t="n">
-        <v>40.4</v>
+        <v>41.1</v>
       </c>
       <c r="Y72" t="n">
         <v>31</v>
@@ -17354,10 +17354,10 @@
         <v>0.031</v>
       </c>
       <c r="W73" t="n">
-        <v>965</v>
+        <v>960</v>
       </c>
       <c r="X73" t="n">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="Y73" t="n">
         <v>27</v>
@@ -17586,7 +17586,7 @@
         <v>0.052</v>
       </c>
       <c r="W74" t="n">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="X74" t="inlineStr"/>
       <c r="Y74" t="n">
@@ -17816,10 +17816,10 @@
         <v>0</v>
       </c>
       <c r="W75" t="n">
-        <v>3819</v>
+        <v>3828</v>
       </c>
       <c r="X75" t="n">
-        <v>86</v>
+        <v>86.2</v>
       </c>
       <c r="Y75" t="n">
         <v>42</v>
@@ -18048,10 +18048,10 @@
         <v>0.006</v>
       </c>
       <c r="W76" t="n">
-        <v>4884</v>
+        <v>4857</v>
       </c>
       <c r="X76" t="n">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="Y76" t="n">
         <v>23</v>
@@ -18276,10 +18276,10 @@
         <v>0.025</v>
       </c>
       <c r="W77" t="n">
-        <v>1581</v>
+        <v>1586</v>
       </c>
       <c r="X77" t="n">
-        <v>38.4</v>
+        <v>38.5</v>
       </c>
       <c r="Y77" t="inlineStr"/>
       <c r="Z77" t="n">
@@ -18496,10 +18496,10 @@
         <v>0</v>
       </c>
       <c r="W78" t="n">
-        <v>31015</v>
+        <v>31208</v>
       </c>
       <c r="X78" t="n">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Y78" t="n">
         <v>62</v>
@@ -18728,7 +18728,7 @@
         <v>0</v>
       </c>
       <c r="W79" t="n">
-        <v>105242</v>
+        <v>105181</v>
       </c>
       <c r="X79" t="n">
         <v>30.3</v>
@@ -18957,10 +18957,10 @@
         </is>
       </c>
       <c r="V80" t="n">
-        <v>0.36</v>
+        <v>0.353</v>
       </c>
       <c r="W80" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="X80" t="inlineStr"/>
       <c r="Y80" t="n">
@@ -19187,13 +19187,13 @@
         </is>
       </c>
       <c r="V81" t="n">
-        <v>0.235</v>
+        <v>0.232</v>
       </c>
       <c r="W81" t="n">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="X81" t="n">
-        <v>22.8</v>
+        <v>22.9</v>
       </c>
       <c r="Y81" t="n">
         <v>21</v>
@@ -19419,10 +19419,10 @@
         </is>
       </c>
       <c r="V82" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="W82" t="n">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="X82" t="inlineStr"/>
       <c r="Y82" t="n">
@@ -21329,31 +21329,31 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TIGERLOGS</t>
+          <t>TRUALT</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Tiger Logistics (India) Limited</t>
+          <t>TRUALT BIOENERGY LIMITED</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>24.27</v>
+        <v>447.2</v>
       </c>
       <c r="D50" t="n">
-        <v>27.53</v>
+        <v>349.57</v>
       </c>
       <c r="E50" t="n">
-        <v>-11.8</v>
+        <v>27.9</v>
       </c>
       <c r="F50" t="n">
-        <v>61.81</v>
+        <v>70.55</v>
       </c>
       <c r="G50" t="n">
-        <v>0.65</v>
+        <v>31.6</v>
       </c>
       <c r="H50" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -21364,140 +21364,140 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TRUALT</t>
+          <t>AVONMORE</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TRUALT BIOENERGY LIMITED</t>
+          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>447.2</v>
+        <v>12.44</v>
       </c>
       <c r="D51" t="n">
-        <v>349.57</v>
+        <v>12.86</v>
       </c>
       <c r="E51" t="n">
-        <v>27.9</v>
+        <v>-3.3</v>
       </c>
       <c r="F51" t="n">
-        <v>70.55</v>
+        <v>69.12</v>
       </c>
       <c r="G51" t="n">
-        <v>31.6</v>
+        <v>2.35</v>
       </c>
       <c r="H51" t="n">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AVONMORE</t>
+          <t>SHAKTIPUMP</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>AVONMORE CAPITAL &amp; MANAGEMENT SERVICES LIMITED</t>
+          <t>SHAKTI PUMPS (INDIA) LIMITED</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>12.44</v>
+        <v>424.45</v>
       </c>
       <c r="D52" t="n">
-        <v>12.86</v>
+        <v>473.17</v>
       </c>
       <c r="E52" t="n">
-        <v>-3.3</v>
+        <v>-10.3</v>
       </c>
       <c r="F52" t="n">
-        <v>69.12</v>
+        <v>56.22</v>
       </c>
       <c r="G52" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
       <c r="H52" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>16-09-2026</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SHAKTIPUMP</t>
+          <t>DANGEE</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SHAKTI PUMPS (INDIA) LIMITED</t>
+          <t>Dangee Dums Limited</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>424.45</v>
+        <v>3.26</v>
       </c>
       <c r="D53" t="n">
-        <v>473.17</v>
+        <v>2.82</v>
       </c>
       <c r="E53" t="n">
-        <v>-10.3</v>
+        <v>15.6</v>
       </c>
       <c r="F53" t="n">
-        <v>56.22</v>
+        <v>64.45</v>
       </c>
       <c r="G53" t="n">
-        <v>2.33</v>
+        <v>2.02</v>
       </c>
       <c r="H53" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>16-09-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DANGEE</t>
+          <t>TIGERLOGS</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Dangee Dums Limited</t>
+          <t>Tiger Logistics (India) Limited</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3.26</v>
+        <v>24.27</v>
       </c>
       <c r="D54" t="n">
-        <v>2.82</v>
+        <v>27.53</v>
       </c>
       <c r="E54" t="n">
-        <v>15.6</v>
+        <v>-11.8</v>
       </c>
       <c r="F54" t="n">
-        <v>64.45</v>
+        <v>61.81</v>
       </c>
       <c r="G54" t="n">
-        <v>2.02</v>
+        <v>0.65</v>
       </c>
       <c r="H54" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
     </row>

</xml_diff>